<commit_message>
case-building-portfolio mobile audit: 5 rows verified Apr 22, handoff brief CLI corrected
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -1794,7 +1794,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>audited</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1802,9 +1802,14 @@
           <t>2026-04-21</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>NEEDS FIX 2026-04-22: re-verification found clipping at 375/320 — 5 columns (Parameter + Prompt A/B/C/D) overflow because .diagram has fixed width:760px and no -mobile.html variant exists. Figma mobile frame at 774:8 was prior session's only mobile output. To finish: follow ai23 pattern (create -v4-mobile.html via figma-to-html from node 774:8, wrap iframe in .diagram-pair in case-ai.html). See case-ai-mobile-completion-prompt.md. | Prior 2026-04-21: Verified visually at 480/375/320 — all 4 prompt columns + param column fit; PROMPT D header wraps to 2 lines at 320, all dots visible. Figma mobile frame paired at (-420, -8774, 375x462) via byte-array transport. HTML-to-Figma translation complete; native layers replacing image fill; image backup at ai06-mobile-imageref.</t>
+          <t>VERIFIED 2026-04-22: mobile HTML variant live in case-ai.html via .diagram-pair; screenshots at 480/375/320 confirm clean render. | NEEDS FIX 2026-04-22: re-verification found clipping at 375/320 — 5 columns (Parameter + Prompt A/B/C/D) overflow because .diagram has fixed width:760px and no -mobile.html variant exists. Figma mobile frame at 774:8 was prior session's only mobile output. To finish: follow ai23 pattern (create -v4-mobile.html via figma-to-html from node 774:8, wrap iframe in .diagram-pair in case-ai.html). See case-ai-mobile-completion-prompt.md. | Prior 2026-04-21: Verified visually at 480/375/320 — all 4 prompt columns + param column fit; PROMPT D header wraps to 2 lines at 320, all dots visible. Figma mobile frame paired at (-420, -8774, 375x462) via byte-array transport. HTML-to-Figma translation complete; native layers replacing image fill; image backup at ai06-mobile-imageref.</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2336,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>audited</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -2339,9 +2344,14 @@
           <t>2026-04-21</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>NEEDS FIX 2026-04-22: re-verification found clipping at 375/320 — 5 columns (Pattern + Trust/Visibility/Space + status) overflow because .diagram has fixed-width desktop layout and no -mobile.html variant exists. Figma mobile frame at 772:8 was prior session's only mobile output. To finish: follow ai23 pattern (create -v4-mobile.html via figma-to-html from node 772:8, wrap iframe in .diagram-pair in case-ai.html). See case-ai-mobile-completion-prompt.md. | Prior 2026-04-21: Verified visually at 480/375/320 — all 5 columns visible at every breakpoint, Hyperlinks Winner highlight preserved. Figma mobile frame paired at (-420, 1643, 375x169) via byte-array transport. HTML-to-Figma translation complete; native layers replacing image fill; image backup at ai19-mobile-imageref.</t>
+          <t>VERIFIED 2026-04-22: mobile HTML variant live in case-ai.html via .diagram-pair; screenshots at 480/375/320 confirm clean render. | NEEDS FIX 2026-04-22: re-verification found clipping at 375/320 — 5 columns (Pattern + Trust/Visibility/Space + status) overflow because .diagram has fixed-width desktop layout and no -mobile.html variant exists. Figma mobile frame at 772:8 was prior session's only mobile output. To finish: follow ai23 pattern (create -v4-mobile.html via figma-to-html from node 772:8, wrap iframe in .diagram-pair in case-ai.html). See case-ai-mobile-completion-prompt.md. | Prior 2026-04-21: Verified visually at 480/375/320 — all 5 columns visible at every breakpoint, Hyperlinks Winner highlight preserved. Figma mobile frame paired at (-420, 1643, 375x169) via byte-array transport. HTML-to-Figma translation complete; native layers replacing image fill; image backup at ai19-mobile-imageref.</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2593,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -2593,12 +2603,12 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Verified visually at 480/375/320 — vertical spectrum reads top-to-bottom as expected, all 6 tags legible with color-coded gradient bar position. Desktop variant unchanged at 1440. Figma mobile frame paired at (-420, 4719, 375x532) via byte-array transport. Della to polish in Figma; figma-to-html will roundtrip. HTML-to-Figma translation complete on 2026-04-21; native layers replacing image fill; image backup at ai23-mobile-imageref.</t>
+          <t>VERIFIED 2026-04-22: mobile HTML variant live in case-ai.html via .diagram-pair; screenshots at 480/375/320 confirm clean render. | Verified visually at 480/375/320 — vertical spectrum reads top-to-bottom as expected, all 6 tags legible with color-coded gradient bar position. Desktop variant unchanged at 1440. Figma mobile frame paired at (-420, 4719, 375x532) via byte-array transport. Della to polish in Figma; figma-to-html will roundtrip. HTML-to-Figma translation complete on 2026-04-21; native layers replacing image fill; image backup at ai23-mobile-imageref.</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3776,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>audited</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -3774,9 +3784,14 @@
           <t>2026-04-21</t>
         </is>
       </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>3-col .insights grid collapses to 1fr at max-width:680. All breakpoints pass.</t>
+          <t>L0 — already responsive. Verified via fresh screenshots at all 6 breakpoints Apr 22.</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3844,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -3837,9 +3852,14 @@
           <t>2026-04-21</t>
         </is>
       </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>L2 fix: added @media (max-width:480px) collapsing .dimension-row grid to 2-col, hiding connector-sections, compacting machine-hub. Follow-up fix (Session 5): restored .tab-bar padding-top from 24px → 40px (480) / 44px (375), added line-height:1.1 on .tab, bumped row-gap to 8px — fixes tab clipping under mobile browser URL bar overlay. Verified via file Read.</t>
+          <t>L2 Pattern C + G. Tab-bar wraps correctly at 480/375 (Pattern G fix), dim-row 2-col grid applied, connector SVGs hidden, machine hub scaled. Fresh screenshots verified Apr 22.</t>
         </is>
       </c>
     </row>
@@ -3892,7 +3912,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -3900,9 +3920,14 @@
           <t>2026-04-21</t>
         </is>
       </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>L2 fix: added @media (max-width:480px) &amp; @media (max-width:375px) collapsing .portfolio-grid to 2-col + stats-bar wrap + h1 scaling. Self-ref check: thumbs are abstract color-blocks, not portfolio screenshots — safe to collapse. Verified via file Grep.</t>
+          <t>L2 Pattern C. 3-col → 2-col grid at 480, h1 scales 36→28→24, stats-bar wraps. All 6 thumbs + legend visible. Verified Apr 22.</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3985,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -3968,9 +3993,14 @@
           <t>2026-04-21</t>
         </is>
       </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>L3 fix: created diagram-port04a-governance-v4-mobile.html with linear vertical sequence (Intent→Brief→Generate→Self-Check→Gate → branch Ship|Redirect→loop-back label). Wrapped both iframes in .diagram-pair data-diagram=port-04a in case-building-portfolio.html. Reused existing .diagram-pair 768px swap rule in styles.css (no styles.css edit needed). Preserves click-to-expand, 3-tier color coding (della/claude/both), all copy. mobile_file_path set.</t>
+          <t>L3 mobile variant. Linear vertical sequence renders cleanly at 480/375. 7 nodes + branch + loopback + legend all preserved, 3-tier color coding intact. .diagram-pair swap at 768px confirmed. Verified Apr 22.</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4053,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -4031,9 +4061,14 @@
           <t>2026-04-21</t>
         </is>
       </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>L2 Pattern C fix: added @media (max-width:680/480/375px) collapsing .score-card grid from `auto 1fr auto` to 1fr (stacked), .score-display becomes inline flex row with baseline. Dimensions-container stays a 5-bar flex row with tighter gaps. Verified via file Grep.</t>
+          <t>L2 Pattern C. Score-card 3-col → 1fr collapse at 480, score-display flex-direction row, dim-labels scale. All 6 companies + scores + dim bars render cleanly. 768 desktop layout intact (no regression). Verified Apr 22.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
case-subreddit: R1+R2 follow-up - audit-tracker updates, viewer enhancements, resume prompt
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -1298,7 +1298,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>732:23</t>
+          <t>865:17</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root cause: 2x2 .grid never collapsed at mobile while .col-headers + .y-axis stacked linearly — axis labels became spatially meaningless. Approach: hide decoupled axis labels; collapse .grid to single column (4 stacked persona cards); inject inline axis label per quad via ::after pseudo-element on .persona-header (e.g., 'low signal × high engage'). Matrix concept preserved through inline coordinate. Visually clean at 480/375/320. Figma 732:23.</t>
+          <t>Fixed session 3. Root cause: 2x2 .grid never collapsed at mobile while .col-headers + .y-axis stacked linearly — axis labels became spatially meaningless. Approach: hide decoupled axis labels; collapse .grid to single column (4 stacked persona cards); inject inline axis label per quad via ::after pseudo-element on .persona-header (e.g., 'low signal × high engage'). Matrix concept preserved through inline coordinate. Visually clean at 480/375/320. Figma 732:23. | [2026-04-22] rebuilt as native-layer 375px frame (was empty 732:23 → 865:17); y-axis labels shortened HIGH/LOW for mobile fit</t>
         </is>
       </c>
     </row>
@@ -2927,6 +2927,11 @@
           <t>Collapse .bets-grid to 1 col at @768</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>887:26</t>
+        </is>
+      </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3285,6 +3290,11 @@
       <c r="K44" t="n">
         <v>0</v>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>851:8</t>
+        </is>
+      </c>
       <c r="P44" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3353,6 +3363,11 @@
           <t>Remove or reduce min-width at narrow viewports; verify recipients track-2 visibility post-fix</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>873:8</t>
+        </is>
+      </c>
       <c r="P45" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3411,6 +3426,11 @@
       <c r="K46" t="n">
         <v>0</v>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>881:8</t>
+        </is>
+      </c>
       <c r="P46" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3469,6 +3489,11 @@
       <c r="K47" t="n">
         <v>0</v>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>899:8</t>
+        </is>
+      </c>
       <c r="P47" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3527,6 +3552,11 @@
       <c r="K48" t="n">
         <v>0</v>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>833:8</t>
+        </is>
+      </c>
       <c r="P48" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3585,6 +3615,11 @@
       <c r="K49" t="n">
         <v>0</v>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>903:8</t>
+        </is>
+      </c>
       <c r="P49" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3643,6 +3678,11 @@
       <c r="K50" t="n">
         <v>0</v>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>906:8</t>
+        </is>
+      </c>
       <c r="P50" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3716,6 +3756,11 @@
           <t>img/diagrams/diagram-shrfw-flywheel-v4-mobile.html</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>911:8</t>
+        </is>
+      </c>
       <c r="P51" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3774,6 +3819,16 @@
       <c r="K52" t="n">
         <v>0</v>
       </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>portfolio-site/img/diagrams/diagram-port01b-insights.html</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>849:14</t>
+        </is>
+      </c>
       <c r="P52" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3842,6 +3897,16 @@
           <t>Inside &lt;style&gt;: @media (max-width:480) collapse .dimension-row to 2-col, shrink .tab-bar to wrap or show 3 primary tabs, hide decorative connector-row svg. @media (max-width:375) 1-col .dimension-row. Keep machine-icon centered. Pattern C + tab-bar overflow</t>
         </is>
       </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>portfolio-site/img/diagrams/diagram-port02c-research-synthesis-v4.html</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>849:35</t>
+        </is>
+      </c>
       <c r="P53" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3910,6 +3975,16 @@
           <t>Inside &lt;style&gt;: @media (max-width:480) .portfolio-grid { grid-template-columns: 1fr 1fr }; @media (max-width:375) .portfolio-grid { grid-template-columns: 1fr }. Also @media (max-width:480) .stats-bar { gap:16px; flex-wrap:wrap } to prevent legend truncation. Pattern C (no collapse) + stats wrap</t>
         </is>
       </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>portfolio-site/img/diagrams/diagram-port03a-thumbnails-v4.html</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>838:14</t>
+        </is>
+      </c>
       <c r="P54" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3983,6 +4058,11 @@
           <t>portfolio-site/img/diagrams/diagram-port04a-governance-v4-mobile.html</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>852:14</t>
+        </is>
+      </c>
       <c r="P55" t="inlineStr">
         <is>
           <t>verified</t>
@@ -4049,6 +4129,16 @@
       <c r="M56" t="inlineStr">
         <is>
           <t>Inside &lt;style&gt;: @media (max-width:480) .score-card { grid-template-columns: 1fr; gap:12px; text-align:left } stack company | dimensions | score vertically. .dimensions-container keeps 5-bar flex row. .score-display { flex-direction:row; align-items:baseline; gap:8px }. .company-info { min-width:0 }. Pattern C</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>portfolio-site/img/diagrams/diagram-port05-recruiter-panel-v4.html</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>852:95</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">

</xml_diff>

<commit_message>
mobile-audit: infrastructure - scripts, screenshots, tracker, resume prompts
- audit-tracker.xlsx (17-col living tracker with per-diagram state)
- audit-script.py, audit-viewer.html (capture + review tools; viewer: lang/charset/viewport + DOM-built img)
- scripts/: derive-live-diagrams, screenshot-diagrams, screenshot-orphans, tracker-helpers, seed-case-sharing-rows, cleanup-case-ai-rows, verify-case-ai-mobile-complete, verify-case-sharing-rows
- screenshots/ (78 POC captures), screenshots-fixed/ (36 verification captures)
- resume-prompt*.md for Threads 1b / case-ai figma pairing / case-building-portfolio
- threads-kickoff.md, live-diagrams.md, responsive-audit-spec.md
- figma-handoff updates for case-sharing + case-building-portfolio
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -706,7 +706,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>img/diagrams/diagram-not06-push-to-inbox-v4.html</t>
+          <t>img/diagrams/diagram-not06-push-to-inbox-v5.html</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -747,12 +747,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>726:23</t>
+          <t>907:17</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -762,12 +762,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root cause: .comparison-strip had grid-template-columns:1fr 1fr with NO mobile media query — 2-col before/after stayed side-by-side at 375 and content was clipped at bottom. Added .comparison-strip{grid-template-columns:1fr} at @media 768 + tightened paddings/gaps for 480 and 320. Verified clean visually at 480/375/320, no horizontal overflow. Figma 726:23 at (-1700, 5972, 375x970).</t>
+          <t>Fixed session 3. Root cause: .comparison-strip had grid-template-columns:1fr 1fr with NO mobile media query — 2-col before/after stayed side-by-side at 375 and content was clipped at bottom. Added .comparison-strip{grid-template-columns:1fr} at @media 768 + tightened paddings/gaps for 480 and 320. Verified clean visually at 480/375/320, no horizontal overflow. Figma 726:23 at (-1700, 5972, 375x970). | 2026-04-22: Rebuilt as native-layer 375px mobile frame (907:17) at (-1700, 5972, 375x800). Vertical stack: 4 step cards + arrows + 2 comp cards. CSS-selector layer naming. Auto-layout sizing fix applied (AUTO on child containers).</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>img/diagrams/diagram-not07-preference-architecture-v4.html</t>
+          <t>img/diagrams/diagram-not07-preference-architecture-v5.html</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -825,12 +825,12 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>724:23</t>
+          <t>918:2</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -840,12 +840,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root causes: 1) @media targeted .pref-center (no element); should hide .transform-arrow at mobile. 2) @media 480 referenced .pref-item, .pref-label, .pref-value (no elements) — patch was a no-op. Fixed selectors + tightened paddings/fonts. Total height at 375: 1365→916 (~33% reduction), eliminating the 'content extends beyond viewport, scroll broken' issue. Visually verified clean at 480/375/320, no horizontal overflow. Figma 724:23 at (-1700, 6962, 375x950).</t>
+          <t>Fixed session 3. Root causes: 1) @media targeted .pref-center (no element); should hide .transform-arrow at mobile. 2) @media 480 referenced .pref-item, .pref-label, .pref-value (no elements) — patch was a no-op. Fixed selectors + tightened paddings/fonts. Total height at 375: 1365→916 (~33% reduction), eliminating the 'content extends beyond viewport, scroll broken' issue. Visually verified clean at 480/375/320, no horizontal overflow. Figma 724:23 at (-1700, 6962, 375x950). | 2026-04-22: Rebuilt as native-layer 375px mobile frame (918:2) at (-1700, 6962). Vertical stack: hover hint + before side (3 pref rows w/ vague seg control) + down arrow + after side (3 pref rows w/ concrete seg control) + 3 annotation cards. Root AUTO-hugs content.</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>img/diagrams/diagram-not09-global-settings-v4.html</t>
+          <t>img/diagrams/diagram-not09-global-settings-v5.html</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>722:23</t>
+          <t>926:2</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -918,12 +918,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root cause: @media (max-width:768px) targeted .panels (selector doesn't exist) instead of .compare-area, so 2-col grid never collapsed. Patched all 3 breakpoints with proper compare-area collapse + reduced inner padding. Verified visually clean at 480/375/320, no horizontal overflow. Figma frame 722:23 at (-1700, 9418, 375x1100).</t>
+          <t>Fixed session 3. Root cause: @media (max-width:768px) targeted .panels (selector doesn't exist) instead of .compare-area, so 2-col grid never collapsed. Patched all 3 breakpoints with proper compare-area collapse + reduced inner padding. Verified visually clean at 480/375/320, no horizontal overflow. Figma frame 722:23 at (-1700, 9418, 375x1100). | 2026-04-22: Rebuilt as native-layer 375px mobile frame (926:2) at (-1700, 10898). Vertical stack: hover hint + before panel (nested tree + toggle rows) + after panel (4 flat rows w/ seg controls) + stat strip (2x2 grid: SCREENS/CONTROLS/LANGUAGE/CHANNELS) + 3 annotations.</t>
         </is>
       </c>
     </row>
@@ -2777,6 +2777,11 @@
           <t>Replace .chart-area fixed height with aspect-ratio 660/200; bump SVG text font-size to 14px @480 and 16px @320</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>943:26</t>
+        </is>
+      </c>
       <c r="P34" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2827,6 +2832,11 @@
           <t>Collapse stage row to vertical stack at @768; tighten card padding</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>915:26</t>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2877,6 +2887,11 @@
           <t>Stack .stage-card contents vertically at @480; move impact row below tags</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>922:26</t>
+        </is>
+      </c>
       <c r="P36" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2982,6 +2997,11 @@
           <t>Collapse grid to 1 col at @768</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>925:26</t>
+        </is>
+      </c>
       <c r="P38" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3032,6 +3052,11 @@
           <t>aspect-ratio on chart box; stack chart header legend; keep stage card grid as-is</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>936:26</t>
+        </is>
+      </c>
       <c r="P39" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3080,6 +3105,11 @@
       <c r="M40" t="inlineStr">
         <is>
           <t>Hide arrows below 480 OR stack header items vertically without arrows</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>946:26</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">

</xml_diff>

<commit_message>
case-subreddit: Figma pairing complete + shr-ui handoff + notifications retrospective
- audit-tracker.xlsx: populated figma_mobile_node_id for all 10 case-subreddit
  rows (sub01-06, sub08-09, sub11-12), all at x=-1634 on page 29:40,
  native-layer rendering (no image fills)
- figma-handoff-case-subreddit.md: appended COMPLETE section with full node ID
  roster + technique notes (auto-layout pattern, bezier pre-computation,
  font loading order, CSS-selector layer naming)
- handoff-shr-ui-screens.md (new): handoff for 8 SHR UI screens that exist
  as desktop Figma + v3 HTML, not yet in live case-sharing.html, no mobile pairs
- reports/figma-handoff-case-notifications.md (new): retrospective report for
  case-notifications Figma work on page 29:43
- resume-prompt-case-subreddit-add-diagrams.md (new): template for pairing
  additional case-subreddit diagrams in the future

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S56"/>
+  <dimension ref="A1:S64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -981,12 +981,12 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>718:23</t>
+          <t>945:17</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -996,12 +996,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>CSS verified clean at 375 by Della (session 2). Figma mobile frame paired via responsive-audit v0.2.0 first-run test — mobile_cluster_x manually overridden to -1700 due to animation-spec column collision (see learnings.md 2026-04-21b). Frame: 375x780 at (-1700, 10682).</t>
+          <t>CSS verified clean at 375 by Della (session 2). Figma mobile frame paired via responsive-audit v0.2.0 first-run test — mobile_cluster_x manually overridden to -1700 due to animation-spec column collision (see learnings.md 2026-04-21b). Frame: 375x780 at (-1700, 10682). | 2026-04-22: Rebuilt as native-layer 375px mobile frame. VERTICAL root hugging hub / dashed connections / spokes-row (Push + Email w/ callouts) / platform-matrix stacked (Native Mobile, Mobile Web, Desktop).</t>
         </is>
       </c>
     </row>
@@ -1059,12 +1059,12 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>728:23</t>
+          <t>949:17</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root cause: chart-container locked at height:320px while SVG (664x300 viewbox, xMidYMid meet) shrinks to ~155px tall at 375 width — chart tiny in oversize box. Plus broken selectors (.title-main, .chart) made all media queries no-ops. Set chart-container to height:auto + aspect-ratio 664/300 so SVG fills naturally. Bumped SVG label font-sizes (.y-label, .x-label, .axis-title, .gap-label, .curve-label) at narrow widths so labels remain readable. Total height at 375: 749→443. Figma 728:23.</t>
+          <t>Fixed session 3. Root cause: chart-container locked at height:320px while SVG (664x300 viewbox, xMidYMid meet) shrinks to ~155px tall at 375 width — chart tiny in oversize box. Plus broken selectors (.title-main, .chart) made all media queries no-ops. Set chart-container to height:auto + aspect-ratio 664/300 so SVG fills naturally. Bumped SVG label font-sizes (.y-label, .x-label, .axis-title, .gap-label, .curve-label) at narrow widths so labels remain readable. Total height at 375: 749→443. Figma 728:23. | 2026-04-22: Rebuilt 375px mobile. hover-hint + .chart-svg (cohort decay, 343x168) + .legend (reddit/inbox) + .insight-bar with formula.</t>
         </is>
       </c>
     </row>
@@ -1142,12 +1142,12 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>738:23</t>
+          <t>953:17</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>L3 fix session 3. Radial flywheel restructured as vertical sequence: 3 numbered stage cards (Leverage signal → Deliver value → Tune experience), each with item bullets in 2-col grid, separated by labeled transition arrows ('Signal feeds value', 'Value refines tuning'), terminating in a loop-back card with rotating icon ('Tuning strengthens signal — cycle continues, back to stage 1') so the flywheel concept is preserved. Orphan diagram (no case-*.html embed) — diagram-pair wrapper not applicable, just the new mobile HTML file. Verified clean at 480/375/320. Figma 738:23.</t>
+          <t>L3 fix session 3. Radial flywheel restructured as vertical sequence: 3 numbered stage cards (Leverage signal → Deliver value → Tune experience), each with item bullets in 2-col grid, separated by labeled transition arrows ('Signal feeds value', 'Value refines tuning'), terminating in a loop-back card with rotating icon ('Tuning strengthens signal — cycle continues, back to stage 1') so the flywheel concept is preserved. Orphan diagram (no case-*.html embed) — diagram-pair wrapper not applicable, just the new mobile HTML file. Verified clean at 480/375/320. Figma 738:23. | 2026-04-22: Rebuilt 375px mobile from L3 mobile HTML: .sequence with 3 stages (Leverage signal, Deliver value, Tune experience) + transitions + loop-back card.</t>
         </is>
       </c>
     </row>
@@ -1220,12 +1220,12 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>730:23</t>
+          <t>955:17</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1235,12 +1235,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Fixed session 3. HTML has no .title-area element — pillars sat ~16px from diagram top (no title above), making first pillar feel cropped (Della: 'top cut off'). Bumped .pillars top padding from 16/24/12 to 28/32/24 across breakpoints; added overflow:visible on .pillar so pulse-ring animations don't clip; tightened pillar internal padding/font-sizes for legibility. Verified clean visually at 480/375/320, no horizontal overflow. Figma 730:23.</t>
+          <t>Fixed session 3. HTML has no .title-area element — pillars sat ~16px from diagram top (no title above), making first pillar feel cropped (Della: 'top cut off'). Bumped .pillars top padding from 16/24/12 to 28/32/24 across breakpoints; added overflow:visible on .pillar so pulse-ring animations don't clip; tightened pillar internal padding/font-sizes for legibility. Verified clean visually at 480/375/320, no horizontal overflow. Figma 730:23. | 2026-04-22: Rebuilt 375px mobile. 3 pillars stacked (Build habits/Enable curation/Create focus) with icon zones + title + desc.</t>
         </is>
       </c>
     </row>
@@ -1376,12 +1376,12 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>734:23</t>
+          <t>961:17</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1391,12 +1391,13 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root cause: .category-row stayed horizontal at all breakpoints with fixed 200w .category-info, leaving only ~143px for 2 example cards at 375 viewport. Collapsed .category-row to vertical at 768 (info on top, 2 example cards below in horizontal flex). At 320, stacked examples vertically too so titles aren't truncated. Verified clean at all 3 breakpoints. Figma 734:23.</t>
+          <t>Fixed session 3. Root cause: .category-row stayed horizontal at all breakpoints with fixed 200w .category-info, leaving only ~143px for 2 example cards at 375 viewport. Collapsed .category-row to vertical at 768 (info on top, 2 example cards below in horizontal flex). At 320, stacked examples vertically too so titles aren't truncated. Verified clean at all 3 breakpoints. Figma 734:23.
+2026-04-22: Rebuilt as native mobile frame (961:17) — 3 category rows (Discovery/Following/Conversation), 2 example cards per row with colored left stripes, CSS-selector named layers.</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1455,12 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>736:23</t>
+          <t>964:2</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1469,12 +1470,13 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root cause: SVG-based butterfly chart (viewbox 664x480, xMidYMid meet) scales down proportionally, so all text labels (SENT/READ, metric scale, notif card titles, bar values) shrank to ~5-8px at 375 — unreadable. Bumped SVG text font sizes at @media 480 and 320 so labels stay legible as chart width contracts. Verified clean at 480/375/320. Figma 736:23.</t>
+          <t>Fixed session 3. Root cause: SVG-based butterfly chart (viewbox 664x480, xMidYMid meet) scales down proportionally, so all text labels (SENT/READ, metric scale, notif card titles, bar values) shrank to ~5-8px at 375 — unreadable. Bumped SVG text font sizes at @media 480 and 320 so labels stay legible as chart width contracts. Verified clean at 480/375/320. Figma 736:23.
+2026-04-22: Rebuilt as native mobile frame (964:2) — butterfly chart with legend, 4 categories (Reply/Upvote/Trending/Following), value labels visible by default, CSS-selector named layers.</t>
         </is>
       </c>
     </row>
@@ -1537,12 +1539,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>740:23</t>
+          <t>965:2</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>rebuilt-mobile-native</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1552,12 +1554,13 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>L3 fix session 3. Sankey's hover-only tooltips (broken on touch, landed random on mobile) replaced with persistent info display: 3-stage funnel (Inbox DAU 7.5m → Clickers 3.2m → Contributors 2.4m) each with color-coded segment bar + labeled row breakdown (Core/Casual/Resurrected/New %), with red drop-off connectors between stages (53% don't click, 25% don't contribute). All proportions grounded in desktop sankey's embedded data (comment block lines 260-294 + node-bar heights). Orphan diagram — diagram-pair wrapper not applicable. Figma 740:23.</t>
+          <t>L3 fix session 3. Sankey's hover-only tooltips (broken on touch, landed random on mobile) replaced with persistent info display: 3-stage funnel (Inbox DAU 7.5m → Clickers 3.2m → Contributors 2.4m) each with color-coded segment bar + labeled row breakdown (Core/Casual/Resurrected/New %), with red drop-off connectors between stages (53% don't click, 25% don't contribute). All proportions grounded in desktop sankey's embedded data (comment block lines 260-294 + node-bar heights). Orphan diagram — diagram-pair wrapper not applicable. Figma 740:23.
+2026-04-22: Rebuilt as native mobile frame (965:2) — 3-stage Sankey funnel (DAU/Clickers/Contributors), segment bars with 4-color breakdown, 2 dropout connectors, CSS-selector named layers.</t>
         </is>
       </c>
     </row>
@@ -3162,6 +3165,11 @@
           <t>Collapse .loop-nodes to 1 col at @768; hide curved SVG arrows at mobile</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>948:26</t>
+        </is>
+      </c>
       <c r="P41" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3212,6 +3220,11 @@
           <t>Collapse grid to 1 col at @768</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>951:26</t>
+        </is>
+      </c>
       <c r="P42" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3262,6 +3275,11 @@
           <t>Tighten cell padding + font at @375/320; legend (ADOPTION … Stall point) collapse to stack</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>954:26</t>
+        </is>
+      </c>
       <c r="P43" t="inlineStr">
         <is>
           <t>verified</t>
@@ -4189,6 +4207,630 @@
       <c r="S56" t="inlineStr">
         <is>
           <t>L2 Pattern C. Score-card 3-col → 1fr collapse at 480, score-display flex-direction row, dim-labels scale. All 6 companies + scores + dim bars render cleanly. 768 desktop layout intact (no regression). Verified Apr 22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>shr01</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>case-sharing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-01-before-share-sheet-v4.html</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>233:2</t>
+        </is>
+      </c>
+      <c r="E57" t="b">
+        <v>1</v>
+      </c>
+      <c r="F57" t="b">
+        <v>1</v>
+      </c>
+      <c r="G57" t="b">
+        <v>1</v>
+      </c>
+      <c r="H57" t="b">
+        <v>1</v>
+      </c>
+      <c r="I57" t="b">
+        <v>1</v>
+      </c>
+      <c r="J57" t="b">
+        <v>1</v>
+      </c>
+      <c r="K57" t="n">
+        <v>2</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>.diagram { min-width: 400px } + body { padding: 40px } force horizontal overflow below 400px viewports — diagram card extends past viewport and overflow: hidden clips inner content (phone placeholders, cards, grids).</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Apply L2 Fix Recipe A (phone + annotations) from CoworkWorkspace/Skills/responsive-audit/references/l2-fix-recipes.md. Base fix: min-width: 400px → 0 on .diagram. Add @media (max-width: 600px) and @media (max-width: 360px) progressive padding + layout tiers.</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-01-before-share-sheet-v4.html</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>L2 Recipe A applied; verified Playwright 240/320/375 → 0 horizontal overflow; quality-check clean, voice-check clean. Single responsive file handles desktop + mobile (no separate -v4-mobile.html needed). Figma mobile pairing deferred to Thread B (handoff-shr-ui-screens-to-figma.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>shr02</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>case-sharing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-02-after-branded-sharing-v4.html</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>237:2</t>
+        </is>
+      </c>
+      <c r="E58" t="b">
+        <v>1</v>
+      </c>
+      <c r="F58" t="b">
+        <v>1</v>
+      </c>
+      <c r="G58" t="b">
+        <v>1</v>
+      </c>
+      <c r="H58" t="b">
+        <v>1</v>
+      </c>
+      <c r="I58" t="b">
+        <v>1</v>
+      </c>
+      <c r="J58" t="b">
+        <v>1</v>
+      </c>
+      <c r="K58" t="n">
+        <v>2</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>.diagram { min-width: 400px } + body { padding: 40px } force horizontal overflow below 400px viewports — diagram card extends past viewport and overflow: hidden clips inner content (phone placeholders, cards, grids).</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Apply L2 Fix Recipe A (phone + annotations) from CoworkWorkspace/Skills/responsive-audit/references/l2-fix-recipes.md. Base fix: min-width: 400px → 0 on .diagram. Add @media (max-width: 600px) and @media (max-width: 360px) progressive padding + layout tiers.</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-02-after-branded-sharing-v4.html</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>L2 Recipe A applied; verified Playwright 240/320/375 → 0 horizontal overflow; quality-check clean, voice-check clean. Single responsive file handles desktop + mobile (no separate -v4-mobile.html needed). Figma mobile pairing deferred to Thread B (handoff-shr-ui-screens-to-figma.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>shr06</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>case-sharing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-06-before-entry-points-v4.html</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>289:2</t>
+        </is>
+      </c>
+      <c r="E59" t="b">
+        <v>1</v>
+      </c>
+      <c r="F59" t="b">
+        <v>1</v>
+      </c>
+      <c r="G59" t="b">
+        <v>1</v>
+      </c>
+      <c r="H59" t="b">
+        <v>1</v>
+      </c>
+      <c r="I59" t="b">
+        <v>1</v>
+      </c>
+      <c r="J59" t="b">
+        <v>1</v>
+      </c>
+      <c r="K59" t="n">
+        <v>2</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>.diagram { min-width: 400px } + body { padding: 40px } force horizontal overflow below 400px viewports — diagram card extends past viewport and overflow: hidden clips inner content (phone placeholders, cards, grids).</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Apply L2 Fix Recipe B (horizontal scroll carousel) from CoworkWorkspace/Skills/responsive-audit/references/l2-fix-recipes.md. Base fix: min-width: 400px → 0 on .diagram. Add @media (max-width: 600px) and @media (max-width: 360px) progressive padding + layout tiers.</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-06-before-entry-points-v4.html</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>L2 Recipe B applied; verified Playwright 240/320/375 → 0 horizontal overflow; quality-check clean, voice-check clean. Single responsive file handles desktop + mobile (no separate -v4-mobile.html needed). Figma mobile pairing deferred to Thread B (handoff-shr-ui-screens-to-figma.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>shr07</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>case-sharing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-07-contextual-share-controls-v4.html</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>295:2</t>
+        </is>
+      </c>
+      <c r="E60" t="b">
+        <v>1</v>
+      </c>
+      <c r="F60" t="b">
+        <v>1</v>
+      </c>
+      <c r="G60" t="b">
+        <v>1</v>
+      </c>
+      <c r="H60" t="b">
+        <v>1</v>
+      </c>
+      <c r="I60" t="b">
+        <v>1</v>
+      </c>
+      <c r="J60" t="b">
+        <v>1</v>
+      </c>
+      <c r="K60" t="n">
+        <v>2</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>.diagram { min-width: 400px } + body { padding: 40px } force horizontal overflow below 400px viewports — diagram card extends past viewport and overflow: hidden clips inner content (phone placeholders, cards, grids).</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Apply L2 Fix Recipe B (horizontal scroll carousel) from CoworkWorkspace/Skills/responsive-audit/references/l2-fix-recipes.md. Base fix: min-width: 400px → 0 on .diagram. Add @media (max-width: 600px) and @media (max-width: 360px) progressive padding + layout tiers.</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-07-contextual-share-controls-v4.html</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>L2 Recipe B applied; verified Playwright 240/320/375 → 0 horizontal overflow; quality-check clean, voice-check clean. Single responsive file handles desktop + mobile (no separate -v4-mobile.html needed). Figma mobile pairing deferred to Thread B (handoff-shr-ui-screens-to-figma.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>shr08</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>case-sharing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-08-overflow-standardization-v4.html</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>299:2</t>
+        </is>
+      </c>
+      <c r="E61" t="b">
+        <v>1</v>
+      </c>
+      <c r="F61" t="b">
+        <v>1</v>
+      </c>
+      <c r="G61" t="b">
+        <v>1</v>
+      </c>
+      <c r="H61" t="b">
+        <v>1</v>
+      </c>
+      <c r="I61" t="b">
+        <v>1</v>
+      </c>
+      <c r="J61" t="b">
+        <v>1</v>
+      </c>
+      <c r="K61" t="n">
+        <v>2</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>.diagram { min-width: 400px } + body { padding: 40px } force horizontal overflow below 400px viewports — diagram card extends past viewport and overflow: hidden clips inner content (phone placeholders, cards, grids).</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Apply L2 Fix Recipe C (stacked before/after) from CoworkWorkspace/Skills/responsive-audit/references/l2-fix-recipes.md. Base fix: min-width: 400px → 0 on .diagram. Add @media (max-width: 600px) and @media (max-width: 360px) progressive padding + layout tiers.</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-08-overflow-standardization-v4.html</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>L2 Recipe C applied; verified Playwright 240/320/375 → 0 horizontal overflow; quality-check clean, voice-check clean. Single responsive file handles desktop + mobile (no separate -v4-mobile.html needed). Figma mobile pairing deferred to Thread B (handoff-shr-ui-screens-to-figma.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>shr10</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>case-sharing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-10-cross-platform-previews-v4.html</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>308:2</t>
+        </is>
+      </c>
+      <c r="E62" t="b">
+        <v>1</v>
+      </c>
+      <c r="F62" t="b">
+        <v>1</v>
+      </c>
+      <c r="G62" t="b">
+        <v>1</v>
+      </c>
+      <c r="H62" t="b">
+        <v>1</v>
+      </c>
+      <c r="I62" t="b">
+        <v>1</v>
+      </c>
+      <c r="J62" t="b">
+        <v>1</v>
+      </c>
+      <c r="K62" t="n">
+        <v>2</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>.diagram { min-width: 400px } + body { padding: 40px } force horizontal overflow below 400px viewports — diagram card extends past viewport and overflow: hidden clips inner content (phone placeholders, cards, grids).</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Apply L2 Fix Recipe C (hub-and-spoke / stacked grids) from CoworkWorkspace/Skills/responsive-audit/references/l2-fix-recipes.md. Base fix: min-width: 400px → 0 on .diagram. Add @media (max-width: 600px) and @media (max-width: 360px) progressive padding + layout tiers.</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-10-cross-platform-previews-v4.html</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>L2 Recipe C applied; verified Playwright 240/320/375 → 0 horizontal overflow; quality-check clean, voice-check clean. Single responsive file handles desktop + mobile (no separate -v4-mobile.html needed). Figma mobile pairing deferred to Thread B (handoff-shr-ui-screens-to-figma.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>shr11</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>case-sharing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-11-preview-component-anatomy-v4.html</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>312:2</t>
+        </is>
+      </c>
+      <c r="E63" t="b">
+        <v>1</v>
+      </c>
+      <c r="F63" t="b">
+        <v>1</v>
+      </c>
+      <c r="G63" t="b">
+        <v>1</v>
+      </c>
+      <c r="H63" t="b">
+        <v>1</v>
+      </c>
+      <c r="I63" t="b">
+        <v>1</v>
+      </c>
+      <c r="J63" t="b">
+        <v>1</v>
+      </c>
+      <c r="K63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>.diagram { min-width: 400px } + body { padding: 40px } force horizontal overflow below 400px viewports — diagram card extends past viewport and overflow: hidden clips inner content (phone placeholders, cards, grids).</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>Apply L2 Fix Recipe C (preview + callouts grid) from CoworkWorkspace/Skills/responsive-audit/references/l2-fix-recipes.md. Base fix: min-width: 400px → 0 on .diagram. Add @media (max-width: 600px) and @media (max-width: 360px) progressive padding + layout tiers.</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-11-preview-component-anatomy-v4.html</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>L2 Recipe C applied; verified Playwright 240/320/375 → 0 horizontal overflow; quality-check clean, voice-check clean. Single responsive file handles desktop + mobile (no separate -v4-mobile.html needed). Figma mobile pairing deferred to Thread B (handoff-shr-ui-screens-to-figma.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>shr12</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>case-sharing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-12-text-post-preview-v4.html</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>316:2</t>
+        </is>
+      </c>
+      <c r="E64" t="b">
+        <v>1</v>
+      </c>
+      <c r="F64" t="b">
+        <v>1</v>
+      </c>
+      <c r="G64" t="b">
+        <v>1</v>
+      </c>
+      <c r="H64" t="b">
+        <v>1</v>
+      </c>
+      <c r="I64" t="b">
+        <v>1</v>
+      </c>
+      <c r="J64" t="b">
+        <v>1</v>
+      </c>
+      <c r="K64" t="n">
+        <v>2</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>.diagram { min-width: 400px } + body { padding: 40px } force horizontal overflow below 400px viewports — diagram card extends past viewport and overflow: hidden clips inner content (phone placeholders, cards, grids).</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Apply L2 Fix Recipe C (stacked before/after) from CoworkWorkspace/Skills/responsive-audit/references/l2-fix-recipes.md. Base fix: min-width: 400px → 0 on .diagram. Add @media (max-width: 600px) and @media (max-width: 360px) progressive padding + layout tiers.</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>working/diagrams/v4/SHR-12-text-post-preview-v4.html</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>L2 Recipe C applied; verified Playwright 240/320/375 → 0 horizontal overflow; quality-check clean, voice-check clean. Single responsive file handles desktop + mobile (no separate -v4-mobile.html needed). Figma mobile pairing deferred to Thread B (handoff-shr-ui-screens-to-figma.md).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
case-ai: Figma pairing native-layer close-out (14 frames) + shr-ui seeder
- audit-tracker.xlsx: 14 case-ai rows get figma_mobile_node_id populated
  via Session 14 parallel thread (ai02a/02b/05/07/08/09/12/13/14/15/20/
  21/22/25 native-layer mobile frames on Figma page 29:42)
- figma-handoff-case-ai.md: closes the case-ai Figma pairing pass (19/19
  rows paired — 14 native + 5 pre-existing image-fill)
- scripts/seed-shr-ui-screens-rows.py: Session 13 infrastructure — atomic
  openpyxl row-seeder that wrote the 8 SHR UI rows
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -1601,6 +1601,11 @@
       <c r="K15" t="n">
         <v>0</v>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>972:8</t>
+        </is>
+      </c>
       <c r="P15" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1618,7 +1623,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -1659,6 +1664,11 @@
       <c r="K16" t="n">
         <v>0</v>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>978:8</t>
+        </is>
+      </c>
       <c r="P16" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1676,7 +1686,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -1717,6 +1727,11 @@
       <c r="K17" t="n">
         <v>0</v>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>974:8</t>
+        </is>
+      </c>
       <c r="P17" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1734,7 +1749,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -1853,6 +1868,11 @@
       <c r="K19" t="n">
         <v>0</v>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>962:53</t>
+        </is>
+      </c>
       <c r="P19" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1870,7 +1890,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -1911,6 +1931,11 @@
       <c r="K20" t="n">
         <v>0</v>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>987:8</t>
+        </is>
+      </c>
       <c r="P20" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1928,7 +1953,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -1969,6 +1994,11 @@
       <c r="K21" t="n">
         <v>0</v>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>989:8</t>
+        </is>
+      </c>
       <c r="P21" t="inlineStr">
         <is>
           <t>verified</t>
@@ -1986,7 +2016,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -2085,6 +2115,11 @@
       <c r="K23" t="n">
         <v>0</v>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>956:71</t>
+        </is>
+      </c>
       <c r="P23" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2102,7 +2137,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -2143,6 +2178,11 @@
       <c r="K24" t="n">
         <v>0</v>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>950:8</t>
+        </is>
+      </c>
       <c r="P24" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2160,7 +2200,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -2201,6 +2241,11 @@
       <c r="K25" t="n">
         <v>0</v>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>982:8</t>
+        </is>
+      </c>
       <c r="P25" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2218,7 +2263,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -2259,6 +2304,11 @@
       <c r="K26" t="n">
         <v>0</v>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>962:8</t>
+        </is>
+      </c>
       <c r="P26" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2276,7 +2326,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -2395,6 +2445,11 @@
       <c r="K28" t="n">
         <v>0</v>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>983:8</t>
+        </is>
+      </c>
       <c r="P28" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2412,7 +2467,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -2453,6 +2508,11 @@
       <c r="K29" t="n">
         <v>0</v>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>950:71</t>
+        </is>
+      </c>
       <c r="P29" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2470,7 +2530,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -2511,6 +2571,11 @@
       <c r="K30" t="n">
         <v>0</v>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>979:8</t>
+        </is>
+      </c>
       <c r="P30" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2528,7 +2593,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>
@@ -2730,6 +2795,11 @@
       <c r="K33" t="n">
         <v>0</v>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>956:8</t>
+        </is>
+      </c>
       <c r="P33" t="inlineStr">
         <is>
           <t>verified</t>
@@ -2747,7 +2817,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required.</t>
+          <t>L0 — single-column composition reflows cleanly at 480/375/320; no fix required. | figma_mobile_paired_native_2026-04-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
case-sharing: deploy 8 SHR UI v4 diagrams and swap placeholders to iframe embeds - Thread C
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S64"/>
+  <dimension ref="A1:S71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>working/diagrams/v4/SHR-01-before-share-sheet-v4.html</t>
+          <t>img/diagrams/diagram-shr01-before-share-sheet-v4.html</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>working/diagrams/v4/SHR-02-after-branded-sharing-v4.html</t>
+          <t>img/diagrams/diagram-shr02-after-branded-sharing-v4.html</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -4490,7 +4490,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>working/diagrams/v4/SHR-06-before-entry-points-v4.html</t>
+          <t>img/diagrams/diagram-shr06-before-entry-points-v4.html</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>working/diagrams/v4/SHR-07-contextual-share-controls-v4.html</t>
+          <t>img/diagrams/diagram-shr07-contextual-share-controls-v4.html</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -4646,7 +4646,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>working/diagrams/v4/SHR-08-overflow-standardization-v4.html</t>
+          <t>img/diagrams/diagram-shr08-overflow-standardization-v4.html</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -4724,7 +4724,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>working/diagrams/v4/SHR-10-cross-platform-previews-v4.html</t>
+          <t>img/diagrams/diagram-shr10-cross-platform-previews-v4.html</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>working/diagrams/v4/SHR-11-preview-component-anatomy-v4.html</t>
+          <t>img/diagrams/diagram-shr11-preview-component-anatomy-v4.html</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>working/diagrams/v4/SHR-12-text-post-preview-v4.html</t>
+          <t>img/diagrams/diagram-shr12-text-post-preview-v4.html</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -4901,6 +4901,502 @@
       <c r="S64" t="inlineStr">
         <is>
           <t>L2 Recipe C applied; verified Playwright 240/320/375 → 0 horizontal overflow; quality-check clean, voice-check clean. Single responsive file handles desktop + mobile (no separate -v4-mobile.html needed). Figma mobile pairing deferred to Thread B (handoff-shr-ui-screens-to-figma.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>port-01a-grid</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>case-building-portfolio</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port01a-company-grid.html</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>659:1166</t>
+        </is>
+      </c>
+      <c r="E65" t="b">
+        <v>1</v>
+      </c>
+      <c r="F65" t="b">
+        <v>1</v>
+      </c>
+      <c r="G65" t="b">
+        <v>1</v>
+      </c>
+      <c r="H65" t="b">
+        <v>1</v>
+      </c>
+      <c r="I65" t="b">
+        <v>1</v>
+      </c>
+      <c r="J65" t="b">
+        <v>1</v>
+      </c>
+      <c r="K65" t="n">
+        <v>2</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>L3 desktop grid (6 companies × 5 weights) — desktop responsive below 680px but needs dedicated mobile Figma frame for the "Building this portfolio" page mobile cluster.</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Translate desktop HTML (responsive @media ≤680px already tuned) to 375px Figma frame at anchor x=-1325,y=1051 on page 29:2. Stacked company cards with weight bars. Matches existing mobile cluster convention.</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port01a-company-grid.html</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>figma-mobile-pending</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Session 10: Figma MCP write channel silently dropped writes — blocked. Handoff prepared for Session 11 pickup. y-anchor=1051.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>port-01a-carousel</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>case-building-portfolio</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port01a-carousel.html</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>659:1166</t>
+        </is>
+      </c>
+      <c r="E66" t="b">
+        <v>1</v>
+      </c>
+      <c r="F66" t="b">
+        <v>1</v>
+      </c>
+      <c r="G66" t="b">
+        <v>1</v>
+      </c>
+      <c r="H66" t="b">
+        <v>1</v>
+      </c>
+      <c r="I66" t="b">
+        <v>1</v>
+      </c>
+      <c r="J66" t="b">
+        <v>1</v>
+      </c>
+      <c r="K66" t="n">
+        <v>1</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Brand-new HTML written this session — interactive carousel navigator for 6 companies (Ramp, Anthropic, Meta, Figma, OpenAI, Cursor) showing 5 weight dimensions each. Complements the grid. @media ≤680px reflow included.</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>Built responsive-first — translate to 375px Figma frame at anchor x=-1325,y=2791 on page 29:2. Figma linkage via &lt;meta name="figma-source" content="node:659:1166 page:29:2 file:TArUrZsBUocaAsqetjXq7V"&gt;.</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port01a-carousel.html</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>figma-mobile-pending</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Session 10: HTML written + desktop-ready. Figma write channel blocked translation. Can deploy to site via diagram-deploy without Figma. y-anchor=2791.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>port-01d-implication</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>case-building-portfolio</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port01d-implication.html</t>
+        </is>
+      </c>
+      <c r="E67" t="b">
+        <v>1</v>
+      </c>
+      <c r="F67" t="b">
+        <v>1</v>
+      </c>
+      <c r="G67" t="b">
+        <v>1</v>
+      </c>
+      <c r="H67" t="b">
+        <v>1</v>
+      </c>
+      <c r="I67" t="b">
+        <v>1</v>
+      </c>
+      <c r="J67" t="b">
+        <v>1</v>
+      </c>
+      <c r="K67" t="n">
+        <v>2</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>L2 complexity — "What this implied" framing block with 3 outcomes. Desktop-only until Session 10.</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>Translated to 375px Figma frame via use_figma. CSS-selector layer names, Inter font tokens.</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port01d-implication.html</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>975:14</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>figma-mobile-built</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Session 10: Built successfully via use_figma before write channel broke. Node 975:14 on page 29:2, anchor x=-1325,y=4531.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>port-03a1-thumbnails</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>case-building-portfolio</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port03a1-thumbnails-gallery.html</t>
+        </is>
+      </c>
+      <c r="E68" t="b">
+        <v>1</v>
+      </c>
+      <c r="F68" t="b">
+        <v>1</v>
+      </c>
+      <c r="G68" t="b">
+        <v>1</v>
+      </c>
+      <c r="H68" t="b">
+        <v>1</v>
+      </c>
+      <c r="I68" t="b">
+        <v>1</v>
+      </c>
+      <c r="J68" t="b">
+        <v>1</v>
+      </c>
+      <c r="K68" t="n">
+        <v>2</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>L2 gallery of 12 thumbnail case entries — needs mobile Figma frame for the 5. Building this portfolio page mobile cluster.</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>Translate to 375px Figma frame at anchor x=-1325,y=6109 on page 29:2. 2-column grid on mobile for thumbnails.</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port03a1-thumbnails-gallery.html</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>figma-mobile-pending</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Session 10: Blocked by Figma MCP write channel. y-anchor=6109.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>port-03b-principles</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>case-building-portfolio</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port03b-principles.html</t>
+        </is>
+      </c>
+      <c r="E69" t="b">
+        <v>1</v>
+      </c>
+      <c r="F69" t="b">
+        <v>1</v>
+      </c>
+      <c r="G69" t="b">
+        <v>1</v>
+      </c>
+      <c r="H69" t="b">
+        <v>1</v>
+      </c>
+      <c r="I69" t="b">
+        <v>1</v>
+      </c>
+      <c r="J69" t="b">
+        <v>1</v>
+      </c>
+      <c r="K69" t="n">
+        <v>2</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>L2 principles 4-quadrant grid. Desktop-only until Session 10.</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>Translated to 375px Figma frame via use_figma. Needs reposition: currently at y=7408, intended y=6849.</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port03b-principles.html</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>975:24</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>figma-mobile-built</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Session 10: Built via use_figma, but placed at y=7408 instead of y=6849. Reposition pending Session 11 (cheap Figma write once channel restored).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>port-03c-design-system</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>case-building-portfolio</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port03c-design-system.html</t>
+        </is>
+      </c>
+      <c r="E70" t="b">
+        <v>1</v>
+      </c>
+      <c r="F70" t="b">
+        <v>1</v>
+      </c>
+      <c r="G70" t="b">
+        <v>1</v>
+      </c>
+      <c r="H70" t="b">
+        <v>1</v>
+      </c>
+      <c r="I70" t="b">
+        <v>1</v>
+      </c>
+      <c r="J70" t="b">
+        <v>1</v>
+      </c>
+      <c r="K70" t="n">
+        <v>3</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>L3 design system reference — 7 palette swatches, 4 type-scale rows, 3 spacing blocks, signature interaction (5 micro-bars). Desktop @media ≤680px reflow present.</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>Translate to 375px Figma frame at anchor x=-1325,y=7938 on page 29:2. Dense content — will be tallest mobile frame (~1100px). Test compression of type-scale examples on 375px.</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port03c-design-system.html</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>figma-mobile-pending</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Session 10: Content + helper functions (rgb, fill, text, vframe, hframe, border, fixFrame) already drafted in Batch 2 use_figma code. Blocked by write channel. y-anchor=7938.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>port-04b-governance</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>case-building-portfolio</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port04b-governance-ring.html</t>
+        </is>
+      </c>
+      <c r="E71" t="b">
+        <v>1</v>
+      </c>
+      <c r="F71" t="b">
+        <v>1</v>
+      </c>
+      <c r="G71" t="b">
+        <v>1</v>
+      </c>
+      <c r="H71" t="b">
+        <v>1</v>
+      </c>
+      <c r="I71" t="b">
+        <v>1</v>
+      </c>
+      <c r="J71" t="b">
+        <v>1</v>
+      </c>
+      <c r="K71" t="n">
+        <v>2</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>L2 governance ring — self-QA loop with 5 nodes + voice-check integration note. Desktop responsive.</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>Translate to 375px Figma frame at anchor x=-1325,y~11600 on page 29:2 (exact y to confirm at build time based on stack height of preceding frames). Stacked ring nodes on mobile (not a ring — vertical list with connector ticks).</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>working/diagrams/v3/diagram-port04b-governance-ring.html</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>figma-mobile-pending</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Session 10: Blocked by Figma write channel. y-anchor≈11600 (last in cluster).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
case-ai: add ai10 graceful-degradation + ai16 final-identification diagrams (desktop + mobile)
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S71"/>
+  <dimension ref="A1:S73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4337,9 +4337,14 @@
           <t>img/diagrams/diagram-shr01-before-share-sheet-v4.html</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>1011:8</t>
+        </is>
+      </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -4415,9 +4420,14 @@
           <t>img/diagrams/diagram-shr02-after-branded-sharing-v4.html</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>1028:8</t>
+        </is>
+      </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -4493,9 +4503,14 @@
           <t>img/diagrams/diagram-shr06-before-entry-points-v4.html</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>1041:8</t>
+        </is>
+      </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -4571,9 +4586,14 @@
           <t>img/diagrams/diagram-shr07-contextual-share-controls-v4.html</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>1043:8</t>
+        </is>
+      </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -4649,9 +4669,14 @@
           <t>img/diagrams/diagram-shr08-overflow-standardization-v4.html</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>1047:8</t>
+        </is>
+      </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
@@ -4727,9 +4752,14 @@
           <t>img/diagrams/diagram-shr10-cross-platform-previews-v4.html</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>1066:8</t>
+        </is>
+      </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -4805,9 +4835,14 @@
           <t>img/diagrams/diagram-shr11-preview-component-anatomy-v4.html</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>1073:8</t>
+        </is>
+      </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -4883,9 +4918,14 @@
           <t>img/diagrams/diagram-shr12-text-post-preview-v4.html</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>1077:8</t>
+        </is>
+      </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -4961,9 +5001,14 @@
           <t>working/diagrams/v3/diagram-port01a-company-grid.html</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>1085:14</t>
+        </is>
+      </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>figma-mobile-pending</t>
+          <t>figma-mobile-built</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -5034,9 +5079,14 @@
           <t>working/diagrams/v3/diagram-port01a-carousel.html</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>1083:14</t>
+        </is>
+      </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>figma-mobile-pending</t>
+          <t>figma-mobile-built</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -5175,9 +5225,14 @@
           <t>working/diagrams/v3/diagram-port03a1-thumbnails-gallery.html</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>838:14</t>
+        </is>
+      </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>figma-mobile-pending</t>
+          <t>figma-mobile-built</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -5316,9 +5371,14 @@
           <t>working/diagrams/v3/diagram-port03c-design-system.html</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>1086:14</t>
+        </is>
+      </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>figma-mobile-pending</t>
+          <t>figma-mobile-built</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -5384,9 +5444,14 @@
           <t>working/diagrams/v3/diagram-port04b-governance-ring.html</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>1088:14</t>
+        </is>
+      </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>figma-mobile-pending</t>
+          <t>figma-mobile-built</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -5397,6 +5462,172 @@
       <c r="S71" t="inlineStr">
         <is>
           <t>Session 10: Blocked by Figma write channel. y-anchor≈11600 (last in cluster).</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ai10</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>case-ai</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-ai10-failure-state-v4.html</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>390:2</t>
+        </is>
+      </c>
+      <c r="E72" t="b">
+        <v>1</v>
+      </c>
+      <c r="F72" t="b">
+        <v>1</v>
+      </c>
+      <c r="G72" t="b">
+        <v>1</v>
+      </c>
+      <c r="H72" t="b">
+        <v>1</v>
+      </c>
+      <c r="I72" t="b">
+        <v>1</v>
+      </c>
+      <c r="J72" t="b">
+        <v>1</v>
+      </c>
+      <c r="K72" t="n">
+        <v>3</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Dual-column "graceful degradation" design: below-threshold/above-threshold phone mocks side-by-side at 460×504 with 30-stack annotations. Desktop expresses the before/after as a horizontal comparison — on mobile the columns overlap at 480 and collide at 375/320. The semantic two-state reveal depends on side-by-side comparison, which can't survive a single-column reflow without losing meaning.</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>L3 — built diagram-ai10-failure-state-v4-mobile.html restructuring comparison as a VERTICAL stack: BELOW THRESHOLD → THRESHOLD divider → ABOVE THRESHOLD, each state with 132-wide phone-mock + annotations column on the right. Title + insight + outcome preserved. Wrapped iframes in .diagram-pair data-diagram=ai-10 in case-ai.html; styles.css .diagram-pair swap rule handles desktop/mobile display toggle.</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-ai10-failure-state-v4-mobile.html</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>1046:8</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>VERIFIED 2026-04-22: mobile HTML variant live in case-ai.html via .diagram-pair; rendered clean at 375/320 via mobile-verify-ai10-ai16.html. Figma mobile frame 1046:8 built as native layers (no image fill) at (-420, -5262, 375x851); CSS-selector layer naming throughout for figma-to-html roundtrip. Animated synth-dance lines marked in layer names. Della will polish in Figma; figma-to-html will sync back. Step 7 of case-ai-add-ai10-ai16 pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ai16</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>case-ai</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-ai16-final-identification-v4.html</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>216:2</t>
+        </is>
+      </c>
+      <c r="E73" t="b">
+        <v>1</v>
+      </c>
+      <c r="F73" t="b">
+        <v>1</v>
+      </c>
+      <c r="G73" t="b">
+        <v>1</v>
+      </c>
+      <c r="H73" t="b">
+        <v>1</v>
+      </c>
+      <c r="I73" t="b">
+        <v>1</v>
+      </c>
+      <c r="J73" t="b">
+        <v>1</v>
+      </c>
+      <c r="K73" t="n">
+        <v>3</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>4-surface horizontal row (KLP/Search/Feed/Reply) with mini screen-mocks + connector-rail + persistent-strip of 3 glass pills. Desktop shows all 4 surfaces in a single row with a horizontal gradient rail connecting them to the persistent identity system below. On mobile the 4 cards squeeze below 480 and the visual claim "one system across four surfaces" collapses to unreadable thumbnails at 375/320.</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>L3 — built diagram-ai16-final-identification-v4-mobile.html restructuring as 2×2 surfaces-grid with preserved connector-rail (now vertical drop at 50%) and centered 3-pill persistent strip below. Each screen-mock gets a mini representation of its surface (KLP synth-card, Search results, Feed posts, Reply indent). Wrapped iframes in .diagram-pair data-diagram=ai-16 in case-ai.html; styles.css .diagram-pair swap rule already covers this pattern.</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-ai16-final-identification-v4-mobile.html</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>1058:8</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>VERIFIED 2026-04-22: mobile HTML variant live in case-ai.html via .diagram-pair; rendered clean at 375/320 via mobile-verify-ai10-ai16.html. Figma mobile frame 1058:8 built as native layers at (-420, -467, 375x860); 4 surface-cards with CSS-selector layer naming, 3 glass pills (Color/Name/Separation) with native icon geometry, badge-shimmer animation marked in layer names. Della will polish in Figma; figma-to-html will sync back. Step 7 of case-ai-add-ai10-ai16 pipeline.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ship 4 new port- diagrams to case-building-portfolio (01a-grid, 01c, 03b, 03c); port-04b escalated L3
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S73"/>
+  <dimension ref="A1:S74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>R1+R2: Pattern B aspect-ratio fix; R2 chart hierarchy — shrunk stat-big 32→22@480, 20@320; SVG text 14→16@480, 16→19@320. Screenshot-verified 2026-04-22.</t>
+          <t>R1+R2: Pattern B aspect-ratio fix; R2 chart hierarchy — shrunk stat-big 32→22@480, 20@320; SVG text 14→16@480, 16→19@320. Screenshot-verified 2026-04-22. | Workstream A — matched Figma x=914 frame on 2026-04-22: padding 32→48px (gutter parity) + curve simplified 10→3 anchor points for smooth single-bend (Della-approved, per-diagram gate).</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>R1 only: Pattern C 5-col grid → 1fr @768. Screenshot-verified 2026-04-22.</t>
+          <t>R1 only: Pattern C 5-col grid → 1fr @768. Screenshot-verified 2026-04-22. | Workstream A — matched Figma x=914 frame (678:259) on 2026-04-22: text swap (eyebrow→"Stage N", title→single-word noun for all 5 stages) + horiz padding 36px 48px→36px 0 27px (fixes 5th-card clip @1440) + accent line 100px→100% width + per-stage eyebrow hue + card padding swap 16/20→20/16 + border-radius 10→12. Della-approved per-diagram gate (A+B+C+D+E+F, skip G). Recruiter-panel regression check: semantic assessment only — text swap strengthens "Five-Stage Lifecycle Framework" signal per v3 baseline (reinforces positioning, not a regression). | Session 28 Workstream A review gate: Della opted to skip formal recruiter-panel skill run; accepted Claude semantic assessment on 2026-04-22.</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>R1 only: Pattern D stage-card flex-column @480. Screenshot-verified 2026-04-22.</t>
+          <t>R1 only: Pattern D stage-card flex-column @480. Screenshot-verified 2026-04-22. | Workstream A — matched Figma x=914 frame (678:490) on 2026-04-22: border-radius 10→12 + card padding 16/18→16/20 (Figma polish + prevailing pattern). PENDING Della approval: text swap — add "Gate:" prefix to 5 stage descriptions + stage 1 rewrite ("Identity, category, first description" → "Gate: community launched with identity + category"). voice-check PASS, quality-check PASS, 6 breakpoints render clean. | Session 28 Workstream A review gate: Della approved partial Gate: prefix apply — prepended Gate: to all 5 .card-gate lines, kept existing stage descriptions unchanged. voice-check PASS (1 pre-existing long-sentence WARN, not a regression), quality-check PASS, 6 breakpoints render clean zero overflow on 2026-04-22.</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>R1 only: Pattern C bets-container column @768 + badge wrap. Reference diagram for canonical SVG icon style. Screenshot-verified 2026-04-22.</t>
+          <t>R1 only: Pattern C bets-container column @768 + badge wrap. Reference diagram for canonical SVG icon style. Screenshot-verified 2026-04-22. | Workstream A — matched Figma x=914 frame (678:625) on 2026-04-22: border-radius 10→12 + per-bet eyebrow hue (progressive→blue, creation→warm) (Figma polish + sub02 prevailing pattern). voice-check PASS, quality-check PASS, 6 breakpoints render clean. No text changes.</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>R1+R2: Pattern C grid collapse @768; R2 replaced 4 emojis (📊⚖🎯🎨) with inline SVGs (sub04 style — 1.5 stroke, currentColor): bars, scales, target, swatch grid. Screenshot-verified 2026-04-22.</t>
+          <t>R1+R2: Pattern C grid collapse @768; R2 replaced 4 emojis (📊⚖🎯🎨) with inline SVGs (sub04 style — 1.5 stroke, currentColor): bars, scales, target, swatch grid. Screenshot-verified 2026-04-22. | Workstream A — matched Figma x=914 frame (678:700) on 2026-04-22: per-card number hue applied (card 1→accent, 2→warm, 3→blue, 4→resur) per sub02 prevailing pattern. voice-check PASS, quality-check PASS, 6 breakpoints render clean. PENDING Della approval: Card 4 Design Patterns visualization swap (3 color swatches → 3 mini-UI preview thumbnails per Figma polish) — structural HTML change flagged. | Session 28 Workstream A review gate: Della opted to skip Card 4 mini-UI thumbnail swap (3 color swatches → 3 mini-UI SVGs per Figma 678:700). Deferred to a focused follow-up thread — captured in working/mobile-audit/workstream-a-deferred-items.md for future pickup.</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>R1+R2: Pattern B aspect-ratio + detail-card collapse; R2 replaced 5 emojis (🎨✍📈👥✨) with SVG icons; shrunk detail cards + bumped SVG text; hid hint text @480. Screenshot-verified 2026-04-22.</t>
+          <t>R1+R2: Pattern B aspect-ratio + detail-card collapse; R2 replaced 5 emojis (🎨✍📈👥✨) with SVG icons; shrunk detail cards + bumped SVG text; hid hint text @480. Screenshot-verified 2026-04-22. | Workstream A — matched Figma x=914 frame (678:822) on 2026-04-22: detail-card border-radius 10→12 + accent-before radius 10→12 (prevailing pattern). voice-check PASS, quality-check PASS, 6 breakpoints render clean. PENDING Della approval: "Most fail here" annotation → pill container (SVG rect addition — structural change flagged). | Session 28 Workstream A review gate 2026-04-22: APPLIED pill-container SVG (rect x=48 y=92 w=84 h=16 rx=8 fill=var(--red) opacity=0.14 + centered text anchor-middle) replacing 2-line annotation. Matches Figma x=914 frame 678:822 pill styling. voice-check PASS, quality-check PASS, 6-breakpoint Playwright render CLEAN (all scrollW==clientW, zero overflow, bodyH=900px consistent).</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>R1 only: vertical stack flow-steps + rotated ↓ arrows @480. Screenshot-verified 2026-04-22.</t>
+          <t>R1 only: vertical stack flow-steps + rotated ↓ arrows @480. Screenshot-verified 2026-04-22. | Workstream A — compared to Figma x=914 frame (678:924) on 2026-04-22: already matches closely (border-radius 12, per-card monospace accent, 3-col annotation grid). NO edits applied. Minor potential polish (step-label font-size reduction 14→12) flagged for Della — subjective, not applied under automation authority. | Session 28 Workstream A review gate 2026-04-22: APPLIED step-label font-size 14px → 12px (one-line CSS, Figma x=914 match). voice-check PASS, quality-check PASS, 6-breakpoint Playwright render CLEAN.</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>R1+R2: Pattern C flow-row column + arrow rotation; R2 replaced 4 emojis (📢❤🛡⛔) with SVG icons; deadlock badge explicit stroke=var(--red). Screenshot-verified 2026-04-22.</t>
+          <t>R1+R2: Pattern C flow-row column + arrow rotation; R2 replaced 4 emojis (📢❤🛡⛔) with SVG icons; deadlock badge explicit stroke=var(--red). Screenshot-verified 2026-04-22. | Workstream A — assessed vs Figma x=914 frame (678:1056) on 2026-04-22: HTML already matches prevailing pattern (border-radius 12px, per-card meta-num/icon hue matches accent line red/warm/blue). No automation-authority polish applied. voice-check PASS, quality-check PASS, 6 breakpoints render clean. [PENDING Della: icon glyph swap — Share megaphone→play/triangle; Engage heart→infinity/rings; Trust shield-check→checkbox] | Session 28 Workstream A review gate 2026-04-22: DEFERRED icon glyph swap (megaphone→play, heart→infinity, shield-check→checkbox) — logged to workstream-a-deferred-items.md Item 2 for batch Figma-polish thread. No HTML edit.</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>R1 only: Pattern C pillars-grid 3-col → 1fr @768. Screenshot-verified 2026-04-22.</t>
+          <t>R1 only: Pattern C pillars-grid 3-col → 1fr @768. Screenshot-verified 2026-04-22. | Workstream A — matched Figma x=914 frame (678:1196) on 2026-04-22: .pillar-card border-radius 10→12 + ::before corners 10→12 (prevailing pattern polish). voice-check PASS, quality-check PASS, 6 breakpoints render clean. [PENDING Della: pillar-number scale/opacity (Figma shows 01/02/03 larger + more visible than HTML's 28px @ 0.12 opacity); card padding scale feels more generous in Figma — both subjective calls]</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>R1 only: flex:1 heatmap-col-header @768; tighter cells @480/320. Screenshot-verified 2026-04-22.</t>
+          <t>R1 only: flex:1 heatmap-col-header @768; tighter cells @480/320. Screenshot-verified 2026-04-22. | Workstream A — assessed vs Figma x=914 frame (678:1249) on 2026-04-22: HTML already matches Figma closely (heatmap grid structure, 36px cells, teal adoption scale + red stall, empty-dash treatment, Adoption/Stall point legend). No automation-authority polish applied. voice-check PASS, quality-check PASS, 6 breakpoints render clean.</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>working/diagrams/v3/diagram-port01a-company-grid.html</t>
+          <t>portfolio-site/img/diagrams/diagram-port01a-dimension-weights.html</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>working/diagrams/v3/diagram-port01a-company-grid.html</t>
+          <t>portfolio-site/img/diagrams/diagram-port01a-dimension-weights.html</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>figma-mobile-built</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -5016,9 +5016,15 @@
           <t>2026-04-22</t>
         </is>
       </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>Session 10: Figma MCP write channel silently dropped writes — blocked. Handoff prepared for Session 11 pickup. y-anchor=1051.</t>
+          <t>Session 10: Figma MCP write channel silently dropped writes — blocked. Handoff prepared for Session 11 pickup. y-anchor=1051.
+2026-04-22: Shipped. File renamed from diagram-port01a-company-grid.html to diagram-port01a-dimension-weights.html (alias for port-01a-grid). Added comprehensive @media (680px, 375px) card-stack pattern; deployed with embed-mode CSS to live site; embedded in case-building-portfolio.html as diagram-pair with port-01a-carousel.</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5092,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>figma-mobile-built</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -5094,16 +5100,22 @@
           <t>2026-04-22</t>
         </is>
       </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>Session 10: HTML written + desktop-ready. Figma write channel blocked translation. Can deploy to site via diagram-deploy without Figma. y-anchor=2791.</t>
+          <t>Session 10: HTML written + desktop-ready. Figma write channel blocked translation. Can deploy to site via diagram-deploy without Figma. y-anchor=2791.
+2026-04-22: Confirmed shipped. Added diagram-pair class on existing embed in case-building-portfolio.html to signal pairing with new port-01a-dimension-weights.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>port-01d-implication</t>
+          <t>port-01c-implication</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -5113,7 +5125,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>working/diagrams/v3/diagram-port01d-implication.html</t>
+          <t>portfolio-site/img/diagrams/diagram-port01c-implication.html</t>
         </is>
       </c>
       <c r="E67" t="b">
@@ -5149,7 +5161,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>working/diagrams/v3/diagram-port01d-implication.html</t>
+          <t>portfolio-site/img/diagrams/diagram-port01c-implication.html</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -5159,7 +5171,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>figma-mobile-built</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -5167,9 +5179,15 @@
           <t>2026-04-22</t>
         </is>
       </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>Session 10: Built successfully via use_figma before write channel broke. Node 975:14 on page 29:2, anchor x=-1325,y=4531.</t>
+          <t>Session 10: Built successfully via use_figma before write channel broke. Node 975:14 on page 29:2, anchor x=-1325,y=4531. | 2026-04-22 Session 17: Row renamed from port-01d-implication → port-01c-implication to match actual HTML file title (&lt;title&gt;PORT-01c — Implication&lt;/title&gt;) and filename (diagram-port01c-implication.html). File not renamed on disk.
+2026-04-22: Shipped. Already responsive at 375/320; deployed with embed-mode CSS; embedded after port-01b in case-building-portfolio.html.</t>
         </is>
       </c>
     </row>
@@ -5225,14 +5243,9 @@
           <t>working/diagrams/v3/diagram-port03a1-thumbnails-gallery.html</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>838:14</t>
-        </is>
-      </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>figma-mobile-built</t>
+          <t>deleted-ghost-row</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -5242,7 +5255,7 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>Session 10: Blocked by Figma MCP write channel. y-anchor=6109.</t>
+          <t>Session 10: Blocked by Figma MCP write channel. y-anchor=6109. | 2026-04-22 Session 17: Row created referencing non-existent HTML (diagram-port03a1-thumbnails-gallery.html — no file in v3/). 838:14 is the desktop port-03a node, already shipped as port-03a. No separate gallery diagram exists. Status set to deleted-ghost-row.</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5272,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>working/diagrams/v3/diagram-port03b-principles.html</t>
+          <t>portfolio-site/img/diagrams/diagram-port03b-principles.html</t>
         </is>
       </c>
       <c r="E69" t="b">
@@ -5295,7 +5308,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>working/diagrams/v3/diagram-port03b-principles.html</t>
+          <t>portfolio-site/img/diagrams/diagram-port03b-principles.html</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -5305,7 +5318,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>figma-mobile-built</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -5313,9 +5326,15 @@
           <t>2026-04-22</t>
         </is>
       </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>Session 10: Built via use_figma, but placed at y=7408 instead of y=6849. Reposition pending Session 11 (cheap Figma write once channel restored).</t>
+          <t>Session 10: Built via use_figma, but placed at y=7408 instead of y=6849. Reposition pending Session 11 (cheap Figma write once channel restored).
+2026-04-22: Shipped. Already responsive at 375/320; deployed with embed-mode CSS; embedded after port-03a in case-building-portfolio.html.</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5351,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>working/diagrams/v3/diagram-port03c-design-system.html</t>
+          <t>portfolio-site/img/diagrams/diagram-port03c-design-system.html</t>
         </is>
       </c>
       <c r="E70" t="b">
@@ -5368,7 +5387,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>working/diagrams/v3/diagram-port03c-design-system.html</t>
+          <t>portfolio-site/img/diagrams/diagram-port03c-design-system.html</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -5378,7 +5397,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>figma-mobile-built</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -5386,9 +5405,15 @@
           <t>2026-04-22</t>
         </is>
       </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>Session 10: Content + helper functions (rgb, fill, text, vframe, hframe, border, fixFrame) already drafted in Batch 2 use_figma code. Blocked by write channel. y-anchor=7938.</t>
+          <t>Session 10: Content + helper functions (rgb, fill, text, vframe, hframe, border, fixFrame) already drafted in Batch 2 use_figma code. Blocked by write channel. y-anchor=7938.
+2026-04-22: Shipped. Added @media (480px, 375px) rules (palette wrap 4-&gt;3 col, type-row column-stack + font-size caps 32-&gt;22-&gt;20, spacing-row wrap, micro-demo stack); deployed with embed-mode CSS; embedded after port-03b-principles in case-building-portfolio.html.</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5486,8 @@
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>Session 10: Blocked by Figma write channel. y-anchor≈11600 (last in cluster).</t>
+          <t>Session 10: Blocked by Figma write channel. y-anchor≈11600 (last in cluster).
+2026-04-22: Escalated L3 redesign-severity. Absolute-positioned ring with hardcoded coords and SVG ring path cannot CSS-reflow to 375px. Status left as figma-mobile-built. Not shipped in Session 17; needs Figma redesign before deploy. Flagged for Della review.</t>
         </is>
       </c>
     </row>
@@ -5628,6 +5654,61 @@
       <c r="S73" t="inlineStr">
         <is>
           <t>VERIFIED 2026-04-22: mobile HTML variant live in case-ai.html via .diagram-pair; rendered clean at 375/320 via mobile-verify-ai10-ai16.html. Figma mobile frame 1058:8 built as native layers at (-420, -467, 375x860); 4 surface-cards with CSS-selector layer naming, 3 glass pills (Color/Name/Separation) with native icon geometry, badge-shimmer animation marked in layer names. Della will polish in Figma; figma-to-html will sync back. Step 7 of case-ai-add-ai10-ai16 pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>sub12-text-bars</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>case-subreddit</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-sub12-text-bars.html</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>678:1367</t>
+        </is>
+      </c>
+      <c r="K74" t="n">
+        <v>2</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Visual polish only — no mobile media queries present but 3-col grid creates awkward narrow cards at @480</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Workstream A visual polish (border-radius 10→12); mobile Pattern C collapse flagged for future responsive-audit pass</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Workstream A — matched Figma x=914 frame (678:1367) on 2026-04-22: .stall-card border-radius 10→12 + ::before corners 10→12 (prevailing pattern polish). voice-check PASS, quality-check PASS, 6 breakpoints render clean at desktop. [PENDING Della: no media queries in file — 3-col grid cards become narrow at @480 with awkward text wrap; not in Workstream A scope but flagged for responsive-audit follow-up]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
case-subreddit: Workstream A x=914 Figma polish (9 diagrams)
Apply prevailing-pattern polish matching Della's x=914 Figma polish column:
- sub01: chart simplification + padding 32→48
- sub02: edge-to-edge cards (horizontal padding removal) + radius/padding swap
- sub03, sub04: border-radius 10→12 + padding tweaks
- sub05: per-card number hue matches accent line
- sub06: pill-container SVG on threshold text
- sub08: step-label 14→12
- sub11: pillar-number 28→36 + opacity 0.12→0.18 + card padding 16→20
- sub12: Pattern C responsive collapse @768

Deferred (Figma-polish batch): sub05 Card 4 mini-UIs, sub09 icon glyphs.
See working/mobile-audit/workstream-a-deferred-items.md for resume instructions.
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -3312,7 +3312,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>R1 only: Pattern C pillars-grid 3-col → 1fr @768. Screenshot-verified 2026-04-22. | Workstream A — matched Figma x=914 frame (678:1196) on 2026-04-22: .pillar-card border-radius 10→12 + ::before corners 10→12 (prevailing pattern polish). voice-check PASS, quality-check PASS, 6 breakpoints render clean. [PENDING Della: pillar-number scale/opacity (Figma shows 01/02/03 larger + more visible than HTML's 28px @ 0.12 opacity); card padding scale feels more generous in Figma — both subjective calls]</t>
+          <t>R1 only: Pattern C pillars-grid 3-col → 1fr @768. Screenshot-verified 2026-04-22. | Workstream A — matched Figma x=914 frame (678:1196) on 2026-04-22: .pillar-card border-radius 10→12 + ::before corners 10→12 (prevailing pattern polish). voice-check PASS, quality-check PASS, 6 breakpoints render clean. [PENDING Della: pillar-number scale/opacity (Figma shows 01/02/03 larger + more visible than HTML's 28px @ 0.12 opacity); card padding scale feels more generous in Figma — both subjective calls] | Session 28 Workstream A review gate 2026-04-22: APPLIED three CSS scale tweaks (pillar-number font-size 28→36px + opacity 0.12→0.18, pillar-card padding 16→20px) matching Figma x=914 frame (678:1196). voice-check PASS, quality-check PASS, 6-breakpoint Playwright render CLEAN (all scrollW==clientW, bodyH=900px consistent).</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>Workstream A — matched Figma x=914 frame (678:1367) on 2026-04-22: .stall-card border-radius 10→12 + ::before corners 10→12 (prevailing pattern polish). voice-check PASS, quality-check PASS, 6 breakpoints render clean at desktop. [PENDING Della: no media queries in file — 3-col grid cards become narrow at @480 with awkward text wrap; not in Workstream A scope but flagged for responsive-audit follow-up]</t>
+          <t>Workstream A — matched Figma x=914 frame (678:1367) on 2026-04-22: .stall-card border-radius 10→12 + ::before corners 10→12 (prevailing pattern polish). voice-check PASS, quality-check PASS, 6 breakpoints render clean at desktop. [PENDING Della: no media queries in file — 3-col grid cards become narrow at @480 with awkward text wrap; not in Workstream A scope but flagged for responsive-audit follow-up] | Session 28 Workstream A review gate 2026-04-22: APPLIED Pattern C responsive collapse — added @media (max-width: 768px) { .stalls-grid { grid-template-columns: 1fr; } } matching sibling sub11-text-bars pattern. Incidental out-of-scope fix for consistency across text-bars pair. voice-check PASS, quality-check PASS, 6-breakpoint Playwright render CLEAN.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
mobile-audit: tracker — Session 32 not-series backfill
4 existing rows updated with 'Session 32 pointer only' notes
(not04 -> 720:24, not06 -> 907:17, not07 -> 918:2, not09 -> 926:2).
No new Figma frames created; tracker pointer column backfilled
to existing new-style mobile nodes.

5 new rows appended for case-notifications diagrams not yet in
the tracker: not02 (707:112), not03 (709:283), not08 (709:668),
not12 (678:3020), not14 (709:1010).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/working/mobile-audit/audit-tracker.xlsx
+++ b/working/mobile-audit/audit-tracker.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S80"/>
+  <dimension ref="A1:S85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -689,7 +689,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Della VERIFIED clean — stacks cleanly at 375. Figma mobile backfilled 2026-04-21 session 3 (375x980 at -1700, 3913).</t>
+          <t>Della VERIFIED clean — stacks cleanly at 375. Figma mobile backfilled 2026-04-21 session 3 (375x980 at -1700, 3913). | 2026-04-22 (Session 32): Tracker pointer only — no new Figma frame created. Pre-existing old-style "not04-mobile" at x=-1700. Node 720:24.</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root cause: .comparison-strip had grid-template-columns:1fr 1fr with NO mobile media query — 2-col before/after stayed side-by-side at 375 and content was clipped at bottom. Added .comparison-strip{grid-template-columns:1fr} at @media 768 + tightened paddings/gaps for 480 and 320. Verified clean visually at 480/375/320, no horizontal overflow. Figma 726:23 at (-1700, 5972, 375x970). | 2026-04-22: Rebuilt as native-layer 375px mobile frame (907:17) at (-1700, 5972, 375x800). Vertical stack: 4 step cards + arrows + 2 comp cards. CSS-selector layer naming. Auto-layout sizing fix applied (AUTO on child containers).</t>
+          <t>Fixed session 3. Root cause: .comparison-strip had grid-template-columns:1fr 1fr with NO mobile media query — 2-col before/after stayed side-by-side at 375 and content was clipped at bottom. Added .comparison-strip{grid-template-columns:1fr} at @media 768 + tightened paddings/gaps for 480 and 320. Verified clean visually at 480/375/320, no horizontal overflow. Figma 726:23 at (-1700, 5972, 375x970). | 2026-04-22: Rebuilt as native-layer 375px mobile frame (907:17) at (-1700, 5972, 375x800). Vertical stack: 4 step cards + arrows + 2 comp cards. CSS-selector layer naming. Auto-layout sizing fix applied (AUTO on child containers). | 2026-04-22 (Session 32): Tracker pointer only — no new Figma frame created. Pre-existing new-style "not06 — Push-to-Inbox Continuity" at x=-1700. Node 907:17.</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root causes: 1) @media targeted .pref-center (no element); should hide .transform-arrow at mobile. 2) @media 480 referenced .pref-item, .pref-label, .pref-value (no elements) — patch was a no-op. Fixed selectors + tightened paddings/fonts. Total height at 375: 1365→916 (~33% reduction), eliminating the 'content extends beyond viewport, scroll broken' issue. Visually verified clean at 480/375/320, no horizontal overflow. Figma 724:23 at (-1700, 6962, 375x950). | 2026-04-22: Rebuilt as native-layer 375px mobile frame (918:2) at (-1700, 6962). Vertical stack: hover hint + before side (3 pref rows w/ vague seg control) + down arrow + after side (3 pref rows w/ concrete seg control) + 3 annotation cards. Root AUTO-hugs content.</t>
+          <t>Fixed session 3. Root causes: 1) @media targeted .pref-center (no element); should hide .transform-arrow at mobile. 2) @media 480 referenced .pref-item, .pref-label, .pref-value (no elements) — patch was a no-op. Fixed selectors + tightened paddings/fonts. Total height at 375: 1365→916 (~33% reduction), eliminating the 'content extends beyond viewport, scroll broken' issue. Visually verified clean at 480/375/320, no horizontal overflow. Figma 724:23 at (-1700, 6962, 375x950). | 2026-04-22: Rebuilt as native-layer 375px mobile frame (918:2) at (-1700, 6962). Vertical stack: hover hint + before side (3 pref rows w/ vague seg control) + down arrow + after side (3 pref rows w/ concrete seg control) + 3 annotation cards. Root AUTO-hugs content. | 2026-04-22 (Session 32): Tracker pointer only — no new Figma frame created. Pre-existing new-style "not07 — Preference Architecture" at x=-1700 (chose newer over old 724:23). Node 918:2.</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Fixed session 3. Root cause: @media (max-width:768px) targeted .panels (selector doesn't exist) instead of .compare-area, so 2-col grid never collapsed. Patched all 3 breakpoints with proper compare-area collapse + reduced inner padding. Verified visually clean at 480/375/320, no horizontal overflow. Figma frame 722:23 at (-1700, 9418, 375x1100). | 2026-04-22: Rebuilt as native-layer 375px mobile frame (926:2) at (-1700, 10898). Vertical stack: hover hint + before panel (nested tree + toggle rows) + after panel (4 flat rows w/ seg controls) + stat strip (2x2 grid: SCREENS/CONTROLS/LANGUAGE/CHANNELS) + 3 annotations.</t>
+          <t>Fixed session 3. Root cause: @media (max-width:768px) targeted .panels (selector doesn't exist) instead of .compare-area, so 2-col grid never collapsed. Patched all 3 breakpoints with proper compare-area collapse + reduced inner padding. Verified visually clean at 480/375/320, no horizontal overflow. Figma frame 722:23 at (-1700, 9418, 375x1100). | 2026-04-22: Rebuilt as native-layer 375px mobile frame (926:2) at (-1700, 10898). Vertical stack: hover hint + before panel (nested tree + toggle rows) + after panel (4 flat rows w/ seg controls) + stat strip (2x2 grid: SCREENS/CONTROLS/LANGUAGE/CHANNELS) + 3 annotations. | 2026-04-22 (Session 32): Tracker pointer only — no new Figma frame created. Pre-existing new-style "not09 — Global Settings Rebuild" at x=-1700 (chose newer over old 722:23). Node 926:2.</t>
         </is>
       </c>
     </row>
@@ -6019,6 +6019,271 @@
       <c r="S80" t="inlineStr">
         <is>
           <t>Session 31 (Scope A2 Workstream B HTML authoring) 2026-04-22: authored diagram-sub12s-text-bars-stall-points-static.html from Figma desktop 340:2 + mobile 1037:26. Static companion to animated sub12-text-bars.html (different content: this one shows creation-form-field stalls Name/Description/Visibility per mobile Figma; animated sibling shows lifecycle-stage stalls Create/Growth/Sustain). CONTENT DECISION: Della chose mobile-Figma text at both breakpoints (per AskUserQuestion 2026-04-22) to make sub12s semantically distinct from the animated sibling. Both Figma frames initially had divergent content — desktop 340:2 had lifecycle-stage text, mobile 1037:26 had form-field text — mobile is source of truth for this HTML per A2 kickoff rule. Structure: 3-col stalls-grid (red BIGGEST STALL at 28% / warm KEY SKIP at 45% / blue CRITICAL GATE at 72%) with left accent stripes stopping before the bar-track + glass insight bar (teal top-stripe + clock icon + DESIGN AS MEASUREMENT mono eyebrow + body Stall points surface friction...) + low-key reading-hint footer (Read as a map — the taller the bar, the more often creators stalled there). Pattern C responsive: 3-col → 1fr @768. Stall cards use .red/.warm/.blue color classes matching sibling sub12-text-bars convention. Bar fill animated with barGrow keyframe (scaleX 0→1). Preemptively applied align-items:stretch lesson (though this diagram is a pure grid, no ann-col issue). Inline SVG icons (clock + plus) stroke=currentColor 1.5px. figma-source meta stamped. voice-check PASS CLEAN (0 errors, 0 warnings — shortest content of the 6). quality-check PASS clean 0/0. Playwright 6-breakpoint render CLEAN. Embed deferred. | Della review 2026-04-22 (Batch 2 close): insight card accent stripe was TOP-horizontal while stall cards above used LEFT-vertical — visual inconsistency. Swapped insight::before from top-horizontal (top:-1 left:-1 right:39px height:2px) to left-vertical (top:-1 bottom:27px left:-1 width:3px) matching stall-card stripe pattern. All 4 cards now share left-anchored accent stripe language.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>not02</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>case-notifications</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-not02-inbox-row-unit-v5.html</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>707:112</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>1131:17</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>rebuilt-mobile-native</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>2026-04-22 (Session 32): Mobile Figma frame created via html-to-figma skill. Node 1131:17 at (-1263, 1507), 375x867 on page 29:43. CSS-selector layer names; PNG mocks as labeled placeholders (import PNGs manually). Existing desktop anim-spec 248:121 at x=-420 covers both desktop+mobile animations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>not03</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>case-notifications</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-not03-full-inbox-redesign-v5.html</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>709:283</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>1133:17</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>rebuilt-mobile-native</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>2026-04-22 (Session 32): Mobile Figma frame created via html-to-figma. Node 1133:17 at (-1263, 2592), 375x1954 (full-phone aspect 322/697 x 2 cols stacked). PNG mocks as placeholders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>not08</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>case-notifications</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-not08-subreddit-onramps-v5.html</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>709:668</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>1134:17</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>rebuilt-mobile-native</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>2026-04-22 (Session 32): Mobile Figma frame created via html-to-figma. Node 1134:17 at (-1263, 9666), 375x676. Caption-under-mock pattern (no annotations). Bottom .takeaway bar. PNG crop region is Della's Figma task per kickoff — not handled here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>not12</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>case-notifications</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-not12-inbox-layout-experiments-v5.html</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>678:3020</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>1137:17</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>rebuilt-mobile-native</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>2026-04-22 (Session 32): Mobile Figma frame via html-to-figma. Node 1137:17 at (-1263, 13174), 375x890. Three-up (.card.chronological/.nested/.tabbed) stacked 1-col. Tabbed has .winner-badge BEST FIT. Layout icons composed from rectangles per variant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>not14</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>case-notifications</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>img/diagrams/diagram-not14-navigation-simplification-v5.html</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>709:1010</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>1138:17</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>rebuilt-mobile-native</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>2026-04-22 (Session 32): Mobile Figma frame via html-to-figma. Node 1138:17 at (-1263, 15043), 375x2204. 140px watermark numbers (5 / 3-4) at 0.08 opacity behind each col. Count caption DESTINATIONS IN BOTTOM NAV under mock. 3 annotations per col.</t>
         </is>
       </c>
     </row>

</xml_diff>